<commit_message>
Adding informal, transport,treatment binaries, adding periods, and weights per person.
</commit_message>
<xml_diff>
--- a/R/Data Cleaning/PLFS_all_column_names_and_labels.xlsx
+++ b/R/Data Cleaning/PLFS_all_column_names_and_labels.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -758,17 +758,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -781,11 +771,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5220,14 +5210,14 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:I160">
-    <cfRule type="containsText" dxfId="2" priority="2" stopIfTrue="1" operator="containsText" text="(NIC)">
-      <formula>NOT(ISERROR(SEARCH("(NIC)",A1)))</formula>
+  <conditionalFormatting sqref="A1:I130">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="(NCO)">
+      <formula>NOT(ISERROR(SEARCH("(NCO)",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:I130">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="(NCO)">
-      <formula>NOT(ISERROR(SEARCH("(NCO)",A1)))</formula>
+  <conditionalFormatting sqref="A1:I160">
+    <cfRule type="containsText" dxfId="0" priority="2" stopIfTrue="1" operator="containsText" text="(NIC)">
+      <formula>NOT(ISERROR(SEARCH("(NIC)",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>